<commit_message>
Change ttests for oneway instead of twoway
</commit_message>
<xml_diff>
--- a/output/t_test_prot_gender.xlsx
+++ b/output/t_test_prot_gender.xlsx
@@ -20,7 +20,7 @@
     <t xml:space="preserve">Mean Female</t>
   </si>
   <si>
-    <t xml:space="preserve">Mean difference</t>
+    <t xml:space="preserve">Mean difference (Male - Female)</t>
   </si>
   <si>
     <t xml:space="preserve">CI lower</t>
@@ -32,7 +32,7 @@
     <t xml:space="preserve">t statistic</t>
   </si>
   <si>
-    <t xml:space="preserve">p value</t>
+    <t xml:space="preserve">p value (one-sided)</t>
   </si>
 </sst>
 </file>
@@ -395,10 +395,10 @@
         <v>22.28</v>
       </c>
       <c r="D2" t="n">
-        <v>20.05</v>
-      </c>
-      <c r="E2" t="n">
-        <v>24.51</v>
+        <v>20.41</v>
+      </c>
+      <c r="E2" t="e">
+        <v>#NUM!</v>
       </c>
       <c r="F2" t="n">
         <v>19.58</v>

</xml_diff>